<commit_message>
v1.1: decision-first research ledger, internal data map, environment kill factor, region/period flags on market values
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/copostly/CoPostly_financial_model.xlsx
+++ b/examples/copostly/CoPostly_financial_model.xlsx
@@ -1985,11 +1985,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="77613928"/>
-        <c:axId val="31439836"/>
+        <c:axId val="49454544"/>
+        <c:axId val="81072924"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="77613928"/>
+        <c:axId val="49454544"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2022,7 +2022,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="31439836"/>
+        <c:crossAx val="81072924"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2030,7 +2030,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="31439836"/>
+        <c:axId val="81072924"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2073,7 +2073,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="77613928"/>
+        <c:crossAx val="49454544"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3371,11 +3371,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="63795004"/>
-        <c:axId val="92168631"/>
+        <c:axId val="527104"/>
+        <c:axId val="21344981"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="63795004"/>
+        <c:axId val="527104"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3408,7 +3408,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="92168631"/>
+        <c:crossAx val="21344981"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3416,7 +3416,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="92168631"/>
+        <c:axId val="21344981"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3459,7 +3459,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="63795004"/>
+        <c:crossAx val="527104"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -4757,11 +4757,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="66602999"/>
-        <c:axId val="29581291"/>
+        <c:axId val="1812577"/>
+        <c:axId val="160818"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="66602999"/>
+        <c:axId val="1812577"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4794,7 +4794,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="29581291"/>
+        <c:crossAx val="160818"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -4802,7 +4802,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="29581291"/>
+        <c:axId val="160818"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4845,7 +4845,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="66602999"/>
+        <c:crossAx val="1812577"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>

</xml_diff>